<commit_message>
Make handing every IP design to the toy factory the first milestone.
Only the HKJC designs have reached the factory. W1 now has our side
finalising all designs (政協青年聯會, and AI Buddy if it ships 1/15) and
a 10/16 milestone: every design delivered, and the factory replies with
a sampling schedule.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/毛公仔打版與量產時間表_草案v0.5.xlsx
+++ b/docs/毛公仔打版與量產時間表_草案v0.5.xlsx
@@ -108,6 +108,15 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -115,15 +124,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -548,7 +548,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="40" customHeight="1">
+    <row r="5" ht="72" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>W1</t>
@@ -561,428 +561,436 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>回覆四個造型的打樣排期</t>
+          <t>收到全部造型後，回覆每個造型的打樣排期</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>交機芯規格；向電路板供應商詢價、追加樣板</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
+          <t>定下全部 IP 造型交玩具廠（目前只交了馬會）；交機芯規格；向電路板供應商詢價、追加樣板</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>10/16 全部造型交工廠</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>馬會兩款、政協青年聯會版、AI Buddy（如 1/15 出貨）的造型圖（正、側、背面，尺寸，顏色）全部交到工廠；工廠回覆打樣排期</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>10/19–10/23</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>機芯盒 3D 設計、第一版初樣</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>審 3D 圖；決定電路板改不改；定好 App 和網頁的對接方式</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
+      <c r="E6" s="9" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr"/>
     </row>
     <row r="7" ht="56" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>10/26–10/30</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>寄出第一版樣品（每款 3 隻）</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>裝板實測，給修改意見；電路板定案</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>10/30 第一版樣品測試</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>收音（1 米）、喇叭響度、按鍵、Wi-Fi、充電、跌落全部測過；修改意見已交工廠</t>
         </is>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>11/2–11/6</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>第二版樣品；機芯盒開模；20 隻測試樣品</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>量產電路板下單；內部測試開始；App 開發</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>11/6 電路板下單</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>3,000 台加備品已下單，供應商確認 12/4 前到廠</t>
         </is>
       </c>
     </row>
     <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>11/9–11/13</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>外觀簽樣；訂面料和配件</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>客戶確認外觀；App 開發</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>11/13 外觀簽樣</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>款式 A 兩個造型、款式 B 由客戶書面簽樣；簽樣品雙方各留一隻</t>
         </is>
       </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>W6</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>11/16–11/20</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>T1 試模；包裝打樣</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>成品送檢（玩具安全、無線、電池）；App 開發</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>11/20 款式 A 兩款數量</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>客戶書面確認兩個造型各多少</t>
         </is>
       </c>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>W7</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>11/23–11/27</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>產前樣；包裝定稿</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>確認產前樣、下大貨單；出廠韌體交電路板供應商；App 測試版</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>11/27 產前樣、大貨單</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>產前樣雙方簽字；大貨單已發出；三個 App 測試版可以安裝使用</t>
         </is>
       </c>
     </row>
     <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>W8</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>11/30–12/4</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>物料和電路板到廠，排產線</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>交燒錄自檢工位和作業指導書；App 提交蘋果和 Google 審核</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>11/30 App 送審</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>三個 App 已提交審核</t>
         </is>
       </c>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>W9</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>12/7–12/11</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>試產 50–100 隻</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>全檢試產品；App 審核（預留被拒重交的時間）</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>12/11 試產、App 過審</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>試產全檢合格，問題已改好；三個 App 通過審核；檢測報告合格</t>
         </is>
       </c>
     </row>
     <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>W10</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>12/14–12/18</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>大貨開始，每日回報產量和不良率</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>App 上架但不公開，客戶驗收</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>12/14 大貨開始</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr"/>
+      <c r="F14" s="5" t="inlineStr"/>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>W11</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>12/21–12/25</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>大貨生產；中期驗貨</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>12/25–26 香港假期</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr"/>
-      <c r="F15" s="5" t="inlineStr"/>
+      <c r="E15" s="9" t="inlineStr"/>
+      <c r="F15" s="8" t="inlineStr"/>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>W12</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>12/28–1/1</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>大貨完成</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>1/1 假期</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>12/31 大貨完成</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>全部數量完成；中期驗貨合格</t>
         </is>
       </c>
     </row>
     <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>W13</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>1/4–1/8</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>緩衝週：返工、補貨；尾期驗貨</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>客戶確認 App 公開日期</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr"/>
-      <c r="F17" s="5" t="inlineStr"/>
+      <c r="E17" s="9" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr"/>
     </row>
     <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>W14</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>1/11–1/15</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>包裝、裝箱、出貨</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>App 公開上架</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>1/15 出貨</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>尾期驗貨合格；出貨清單和序號／MAC 對照表；每台已在系統登記</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>W15–16</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>1/18–1/29</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr"/>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr"/>
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>運送、簽收</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>1/29 送達</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>全部簽收</t>
         </is>
@@ -1070,157 +1078,157 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>收音</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>距離 1 米正常說話，語音識別正確；和裸板比較不能明顯變差</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr"/>
-      <c r="D2" s="4" t="inlineStr"/>
-      <c r="E2" s="4" t="inlineStr"/>
-      <c r="F2" s="4" t="inlineStr"/>
-      <c r="G2" s="4" t="inlineStr"/>
+      <c r="C2" s="7" t="inlineStr"/>
+      <c r="D2" s="7" t="inlineStr"/>
+      <c r="E2" s="7" t="inlineStr"/>
+      <c r="F2" s="7" t="inlineStr"/>
+      <c r="G2" s="7" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>喇叭</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>隔著布料的響度和清晰度；最大音量不破音、不震動</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr"/>
-      <c r="D3" s="4" t="inlineStr"/>
-      <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="4" t="inlineStr"/>
-      <c r="G3" s="4" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>按鍵</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>隔著布料／徽章按得到，小朋友按得動，回彈清楚</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr"/>
-      <c r="E4" s="4" t="inlineStr"/>
-      <c r="F4" s="4" t="inlineStr"/>
-      <c r="G4" s="4" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Wi-Fi</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>裝進公仔後訊號強度，和裸板比較</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="4" t="inlineStr"/>
-      <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="4" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>充電</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>USB-C 插得進，充電時燈號看得到</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="4" t="inlineStr"/>
-      <c r="E6" s="4" t="inlineStr"/>
-      <c r="F6" s="4" t="inlineStr"/>
-      <c r="G6" s="4" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>燈號</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>低電紅燈從外面看得到（或確定不外露）</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr"/>
-      <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="4" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>跌落</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>1 米跌落，零件不脫落，機芯盒不鬆脫</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="4" t="inlineStr"/>
-      <c r="E8" s="4" t="inlineStr"/>
-      <c r="F8" s="4" t="inlineStr"/>
-      <c r="G8" s="4" t="inlineStr"/>
+      <c r="C8" s="7" t="inlineStr"/>
+      <c r="D8" s="7" t="inlineStr"/>
+      <c r="E8" s="7" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr"/>
+      <c r="G8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>小零件與尖角</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>眼睛、徽章、配件拉力測試；沒有尖角和可吞食的小零件</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="4" t="inlineStr"/>
-      <c r="E9" s="4" t="inlineStr"/>
-      <c r="F9" s="4" t="inlineStr"/>
-      <c r="G9" s="4" t="inlineStr"/>
+      <c r="C9" s="7" t="inlineStr"/>
+      <c r="D9" s="7" t="inlineStr"/>
+      <c r="E9" s="7" t="inlineStr"/>
+      <c r="F9" s="7" t="inlineStr"/>
+      <c r="G9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>拆裝</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>機芯盒能取出維修，縫口或拉鍊位置合理</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="4" t="inlineStr"/>
-      <c r="F10" s="4" t="inlineStr"/>
-      <c r="G10" s="4" t="inlineStr"/>
+      <c r="C10" s="7" t="inlineStr"/>
+      <c r="D10" s="7" t="inlineStr"/>
+      <c r="E10" s="7" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr"/>
+      <c r="G10" s="7" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Give the apps their own milestones and acceptance criteria.
A new 'App 開發與上架' sheet in the factory workbook, and a matching table
in roadmap.md, list nine app milestones from the bridge spec (10/23) to
public release (1/15), each with checkable criteria: in-app login and
deletion, Bluetooth setup within 10 minutes on iPhone and Android, the
full install-to-unbind flow on two phones per platform, clear error
messages, push, store listing materials, review, and client sign-off.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/毛公仔打版與量產時間表_草案v0.5.xlsx
+++ b/docs/毛公仔打版與量產時間表_草案v0.5.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="時間表" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="樣品測試項目" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App 開發與上架" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="樣品測試項目" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'時間表'!$4:$4</definedName>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,6 +56,12 @@
       <b val="1"/>
       <color rgb="0017202B"/>
       <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <b val="1"/>
+      <color rgb="0017202B"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="4">
@@ -101,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -126,6 +133,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -856,7 +864,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr"/>
     </row>
-    <row r="15" ht="24" customHeight="1">
+    <row r="15" ht="40" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>W11</t>
@@ -968,7 +976,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="24" customHeight="1">
+    <row r="19" ht="40" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>W15–16</t>
@@ -1023,6 +1031,281 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>App 開發與上架：里程碑和驗收標準</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>網頁 App 包在原生殼裡，三個品牌各一個 App。殼過審後，網頁畫面可以繼續更新，不用重新送審。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>週次</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>里程碑</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>驗收標準（全部做到才算完成）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="72" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>10/23</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>對接方案定案</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>① 網頁和殼的對接清單：藍牙配網、原生登入、推送、麥克風、刪除帳號、深層連結，每項寫明介面、參數、回傳和錯誤
+② 做殼的同事書面確認
+③ 三個 App 的名稱、圖示、bundle id 定好</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>10/30</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>登入和品牌主題</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>① email 驗證碼登入可用；Google／Apple 登入由殼完成，網頁收得到登入結果
+② App 內可以刪除帳號
+③ 三個品牌各自的顏色、logo、文案顯示正確，畫面不閃</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>11/6</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>AI Buddy App 可以內部測試</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>① iPhone 和 Android 都能用藍牙找到玩具、選 Wi-Fi、完成綁定，10 分鐘內做完
+② 選角色、對話、改設定、解綁都正常
+③ 家長控制（家長鎖、每日上限）可用</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="56" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>11/20</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>快活和政協青年聯會 App 頁面完成</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>① 快活：會員綁定、查看記憶、一鍵忘記、選語言（粵／普／英）
+② 政協青年聯會版：品牌頁面和角色
+③ 三個 App 都有測試版可以安裝（TestFlight、Google 內部測試）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="88" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>11/27</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>功能凍結</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>① 三個 App 全流程通過：安裝 → 登入 → 藍牙配網 → 綁定 → 對話 → 解綁；iOS 和 Android 各至少兩款手機
+② Wi-Fi 密碼錯、玩具已被別人綁定、斷網時都有清楚提示
+③ 推送收得到：玩具第一次上線、低電提醒
+④ 連續使用 30 分鐘不閃退</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="56" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>11/30</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>提交商店審核</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>① 上架資料齊全：截圖、描述、私隱政策網址、私隱標籤、審核用測試帳號、玩具示範影片
+② 三個 App 已提交蘋果和 Google</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>12/11</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>通過審核</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>① 三個 App 都通過蘋果和 Google 審核
+② 如果被拒，修改後重交並通過</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="56" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>W10</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>12/18</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>客戶驗收</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>① 馬會、政協青年聯會用正式版走一次完整流程，書面確認
+② 找 3 位非團隊成員，從開箱到第一次對話都在 10 分鐘內完成
+③ App 已上架但不公開</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>公開上架</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>① 三個 App 公開，用戶搜尋得到
+② App 內看得到客服聯絡方式、常見問題、保修條款</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Highlight only the milestone and acceptance cells in the factory timeline.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/毛公仔打版與量產時間表_草案v0.5.xlsx
+++ b/docs/毛公仔打版與量產時間表_草案v0.5.xlsx
@@ -108,26 +108,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -582,35 +579,35 @@
           <t>10/16 全部造型交工廠</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>馬會兩款、政協青年聯會版、AI Buddy（如 1/15 出貨）的造型圖（正、側、背面，尺寸，顏色）全部交到工廠；工廠回覆打樣排期</t>
         </is>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>10/19–10/23</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>機芯盒 3D 設計、第一版初樣</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>審 3D 圖；決定電路板改不改；定好 App 和網頁的對接方式</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr"/>
+      <c r="E6" s="8" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="56" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -638,7 +635,7 @@
           <t>10/30 第一版樣品測試</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>收音（1 米）、喇叭響度、按鍵、Wi-Fi、充電、跌落全部測過；修改意見已交工廠</t>
         </is>
@@ -670,7 +667,7 @@
           <t>11/6 電路板下單</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>3,000 台加備品已下單，供應商確認 12/4 前到廠</t>
         </is>
@@ -702,7 +699,7 @@
           <t>11/13 外觀簽樣</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>款式 A 兩個造型、款式 B 由客戶書面簽樣；簽樣品雙方各留一隻</t>
         </is>
@@ -734,7 +731,7 @@
           <t>11/20 款式 A 兩款數量</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>客戶書面確認兩個造型各多少</t>
         </is>
@@ -766,7 +763,7 @@
           <t>11/27 產前樣、大貨單</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>產前樣雙方簽字；大貨單已發出；三個 App 測試版可以安裝使用</t>
         </is>
@@ -798,7 +795,7 @@
           <t>11/30 App 送審</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>三個 App 已提交審核</t>
         </is>
@@ -830,7 +827,7 @@
           <t>12/11 試產、App 過審</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>試產全檢合格，問題已改好；三個 App 通過審核；檢測報告合格</t>
         </is>
@@ -862,31 +859,31 @@
           <t>12/14 大貨開始</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr"/>
+      <c r="F14" s="7" t="inlineStr"/>
     </row>
     <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>W11</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>12/21–12/25</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>大貨生產；中期驗貨</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>12/25–26 香港假期</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr"/>
-      <c r="F15" s="8" t="inlineStr"/>
+      <c r="E15" s="8" t="inlineStr"/>
+      <c r="F15" s="5" t="inlineStr"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
@@ -914,35 +911,35 @@
           <t>12/31 大貨完成</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>全部數量完成；中期驗貨合格</t>
         </is>
       </c>
     </row>
     <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>W13</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>1/4–1/8</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>緩衝週：返工、補貨；尾期驗貨</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>客戶確認 App 公開日期</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr"/>
-      <c r="F17" s="8" t="inlineStr"/>
+      <c r="E17" s="8" t="inlineStr"/>
+      <c r="F17" s="5" t="inlineStr"/>
     </row>
     <row r="18" ht="40" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
@@ -970,7 +967,7 @@
           <t>1/15 出貨</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>尾期驗貨合格；出貨清單和序號／MAC 對照表；每台已在系統登記</t>
         </is>
@@ -998,7 +995,7 @@
           <t>1/29 送達</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>全部簽收</t>
         </is>
@@ -1007,7 +1004,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>黃色行是關鍵節點：延誤的話，後面的日期會跟著推遲，請提早通知。</t>
+          <t>黃色格是關鍵節點和驗收標準：延誤的話，後面的日期會跟著推遲，請提早通知。</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1043,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>App 開發與上架：里程碑和驗收標準</t>
         </is>
@@ -1082,22 +1079,22 @@
       </c>
     </row>
     <row r="5" ht="72" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>10/23</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>對接方案定案</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>① 網頁和殼的對接清單：藍牙配網、原生登入、推送、麥克風、刪除帳號、深層連結，每項寫明介面、參數、回傳和錯誤
 ② 做殼的同事書面確認
@@ -1106,22 +1103,22 @@
       </c>
     </row>
     <row r="6" ht="72" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>10/30</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>登入和品牌主題</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>① email 驗證碼登入可用；Google／Apple 登入由殼完成，網頁收得到登入結果
 ② App 內可以刪除帳號
@@ -1130,22 +1127,22 @@
       </c>
     </row>
     <row r="7" ht="72" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>11/6</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>AI Buddy App 可以內部測試</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>① iPhone 和 Android 都能用藍牙找到玩具、選 Wi-Fi、完成綁定，10 分鐘內做完
 ② 選角色、對話、改設定、解綁都正常
@@ -1154,22 +1151,22 @@
       </c>
     </row>
     <row r="8" ht="56" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>W6</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>11/20</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>快活和政協青年聯會 App 頁面完成</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>① 快活：會員綁定、查看記憶、一鍵忘記、選語言（粵／普／英）
 ② 政協青年聯會版：品牌頁面和角色
@@ -1178,22 +1175,22 @@
       </c>
     </row>
     <row r="9" ht="88" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>W7</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>11/27</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>功能凍結</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>① 三個 App 全流程通過：安裝 → 登入 → 藍牙配網 → 綁定 → 對話 → 解綁；iOS 和 Android 各至少兩款手機
 ② Wi-Fi 密碼錯、玩具已被別人綁定、斷網時都有清楚提示
@@ -1203,22 +1200,22 @@
       </c>
     </row>
     <row r="10" ht="56" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>W8</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>11/30</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>提交商店審核</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>① 上架資料齊全：截圖、描述、私隱政策網址、私隱標籤、審核用測試帳號、玩具示範影片
 ② 三個 App 已提交蘋果和 Google</t>
@@ -1226,22 +1223,22 @@
       </c>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>W9</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>12/11</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>通過審核</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>① 三個 App 都通過蘋果和 Google 審核
 ② 如果被拒，修改後重交並通過</t>
@@ -1249,22 +1246,22 @@
       </c>
     </row>
     <row r="12" ht="56" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>W10</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>12/18</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>客戶驗收</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>① 馬會、政協青年聯會用正式版走一次完整流程，書面確認
 ② 找 3 位非團隊成員，從開箱到第一次對話都在 10 分鐘內完成
@@ -1273,22 +1270,22 @@
       </c>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>W14</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>1/15</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>公開上架</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>① 三個 App 公開，用戶搜尋得到
 ② App 內看得到客服聯絡方式、常見問題、保修條款</t>
@@ -1361,157 +1358,157 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>收音</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>距離 1 米正常說話，語音識別正確；和裸板比較不能明顯變差</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr"/>
-      <c r="D2" s="7" t="inlineStr"/>
-      <c r="E2" s="7" t="inlineStr"/>
-      <c r="F2" s="7" t="inlineStr"/>
-      <c r="G2" s="7" t="inlineStr"/>
+      <c r="C2" s="4" t="inlineStr"/>
+      <c r="D2" s="4" t="inlineStr"/>
+      <c r="E2" s="4" t="inlineStr"/>
+      <c r="F2" s="4" t="inlineStr"/>
+      <c r="G2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>喇叭</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>隔著布料的響度和清晰度；最大音量不破音、不震動</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
+      <c r="C3" s="4" t="inlineStr"/>
+      <c r="D3" s="4" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr"/>
+      <c r="F3" s="4" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>按鍵</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>隔著布料／徽章按得到，小朋友按得動，回彈清楚</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Wi-Fi</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>裝進公仔後訊號強度，和裸板比較</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>充電</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>USB-C 插得進，充電時燈號看得到</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>燈號</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>低電紅燈從外面看得到（或確定不外露）</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
+      <c r="C7" s="4" t="inlineStr"/>
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>跌落</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>1 米跌落，零件不脫落，機芯盒不鬆脫</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr"/>
-      <c r="D8" s="7" t="inlineStr"/>
-      <c r="E8" s="7" t="inlineStr"/>
-      <c r="F8" s="7" t="inlineStr"/>
-      <c r="G8" s="7" t="inlineStr"/>
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr"/>
+      <c r="F8" s="4" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>小零件與尖角</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>眼睛、徽章、配件拉力測試；沒有尖角和可吞食的小零件</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr"/>
-      <c r="D9" s="7" t="inlineStr"/>
-      <c r="E9" s="7" t="inlineStr"/>
-      <c r="F9" s="7" t="inlineStr"/>
-      <c r="G9" s="7" t="inlineStr"/>
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>拆裝</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>機芯盒能取出維修，縫口或拉鍊位置合理</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr"/>
-      <c r="D10" s="7" t="inlineStr"/>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr"/>
-      <c r="G10" s="7" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Give the toy factory and our side each their own acceptance column.
The factory timeline now reads week, dates, key milestone, toy factory,
its acceptance criteria, our side, our acceptance criteria, so each
check sits next to the task it verifies. Every week has criteria for
both sides; only the milestone and acceptance cells are yellow.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/毛公仔打版與量產時間表_草案v0.5.xlsx
+++ b/docs/毛公仔打版與量產時間表_草案v0.5.xlsx
@@ -118,10 +118,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -496,15 +496,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -534,26 +535,31 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>關鍵節點</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
           <t>玩具廠</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>驗收標準（玩具廠）</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>我方（電路板、韌體、App）</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>關鍵節點</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>驗收標準</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="72" customHeight="1">
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>驗收標準（我方）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="88" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>W1</t>
@@ -566,26 +572,31 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
+          <t>10/16 全部造型交工廠</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
           <t>收到全部造型後，回覆每個造型的打樣排期</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>書面打樣排期表：每個造型的初樣和第一版樣品日期</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>定下全部 IP 造型交玩具廠（目前只交了馬會）；交機芯規格；向電路板供應商詢價、追加樣板</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>10/16 全部造型交工廠</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>馬會兩款、政協青年聯會版、AI Buddy（如 1/15 出貨）的造型圖（正、側、背面，尺寸，顏色）全部交到工廠；工廠回覆打樣排期</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1">
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>馬會兩款、政協青年聯會版、AI Buddy（如 1/15 出貨）的造型圖（正、側、背面，尺寸，顏色）和機芯規格全部交到工廠；50 片樣板已下單</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="56" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>W2</t>
@@ -596,20 +607,29 @@
           <t>10/19–10/23</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr"/>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>機芯盒 3D 設計、第一版初樣</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>機芯盒 3D 圖和每個造型的初樣照片交我方</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>審 3D 圖；決定電路板改不改；定好 App 和網頁的對接方式</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-    </row>
-    <row r="7" ht="56" customHeight="1">
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>2 個工作天內回覆 3D 圖意見；改不改板有書面結論；對接清單由做殼的同事確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>W3</t>
@@ -622,26 +642,31 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
+          <t>10/30 第一版樣品測試</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
           <t>寄出第一版樣品（每款 3 隻）</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>裝板實測，給修改意見；電路板定案</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>10/30 第一版樣品測試</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>收音（1 米）、喇叭響度、按鍵、Wi-Fi、充電、跌落全部測過；修改意見已交工廠</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="40" customHeight="1">
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>按「樣品測試項目」自檢後寄出，10/28 前送到我方</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>裝板實測，給修改意見；電路板定案；App 登入和品牌主題</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>收音、喇叭響度、按鍵、Wi-Fi、充電、跌落全部測過，修改意見 10/30 前交工廠；電路板連續對話 2 小時不當機</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="88" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>W4</t>
@@ -654,26 +679,31 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
+          <t>11/6 電路板下單</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
           <t>第二版樣品；機芯盒開模；20 隻測試樣品</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>量產電路板下單；內部測試開始；App 開發</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>11/6 電路板下單</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>3,000 台加備品已下單，供應商確認 12/4 前到廠</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1">
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>第二版改好上一輪全部意見；開模排期確認；20 隻測試樣品交我方</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>量產電路板下單；內部測試開始；AI Buddy App 可以內部測試</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>3,000 台加備品已下單，供應商確認 12/4 前到廠；20 台內部測試機在用；AI Buddy App 在 iPhone、Android 上 10 分鐘內完成配網和綁定</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="56" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>W5</t>
@@ -686,26 +716,31 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
+          <t>11/13 外觀簽樣</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
           <t>外觀簽樣；訂面料和配件</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>客戶確認外觀；App 開發</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>11/13 外觀簽樣</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>款式 A 兩個造型、款式 B 由客戶書面簽樣；簽樣品雙方各留一隻</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="40" customHeight="1">
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>簽樣品雙方各留一隻；長交期物料已下單，交期在 12/4 前</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>客戶確認外觀；出廠韌體底層凍結</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>款式 A 兩個造型、款式 B 由客戶書面簽樣；分區表和加密流程凍結</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="56" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>W6</t>
@@ -718,26 +753,31 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
+          <t>11/20 款式 A 兩款數量</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
           <t>T1 試模；包裝打樣</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>成品送檢（玩具安全、無線、電池）；App 開發</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>11/20 款式 A 兩款數量</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>客戶書面確認兩個造型各多少</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="40" customHeight="1">
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>T1 機芯盒裝得進電路板、電池、喇叭，按鍵和開孔位置正確；包裝打樣交我方</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>成品送檢；快活和政協青年聯會 App 頁面</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>玩具安全、無線、電池已送檢；客戶書面確認款式 A 兩款各多少；三個 App 有可以安裝的測試版</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="56" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>W7</t>
@@ -750,26 +790,31 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
+          <t>11/27 產前樣、大貨單</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
           <t>產前樣；包裝定稿</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>確認產前樣、下大貨單；出廠韌體交電路板供應商；App 測試版</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>11/27 產前樣、大貨單</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>產前樣雙方簽字；大貨單已發出；三個 App 測試版可以安裝使用</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="40" customHeight="1">
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>產前樣和簽樣品一致，「樣品測試項目」全部合格；包裝稿雙方確認</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>確認產前樣、下大貨單；出廠韌體交電路板供應商；App 功能凍結</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>產前樣雙方簽字；大貨單已發出；出廠韌體已交；三個 App 全流程在 iOS、Android 各兩款手機通過</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="56" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>W8</t>
@@ -782,26 +827,31 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
+          <t>11/30 App 送審</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
           <t>物料和電路板到廠，排產線</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>物料和電路板點數無缺；生產排期表交我方</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>交燒錄自檢工位和作業指導書；App 提交蘋果和 Google 審核</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>11/30 App 送審</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>三個 App 已提交審核</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="40" customHeight="1">
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>工位在工廠試跑 10 台全部通過；三個 App 已提交，上架資料齊全</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="56" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>W9</t>
@@ -814,26 +864,31 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
+          <t>12/11 試產、App 過審</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
           <t>試產 50–100 隻</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>全檢合格，發現的問題已改好</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>全檢試產品；App 審核（預留被拒重交的時間）</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>12/11 試產、App 過審</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>試產全檢合格，問題已改好；三個 App 通過審核；檢測報告合格</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="40" customHeight="1">
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>試產品配網、對話、充電全部測過；三個 App 通過審核；檢測報告合格</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="56" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>W10</t>
@@ -846,20 +901,29 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>大貨開始，每日回報產量和不良率</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
+          <t>12/14 大貨開始</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>大貨開始</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>每天回報產量和不良率</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>App 上架但不公開，客戶驗收</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>12/14 大貨開始</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr"/>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>客戶書面確認 App；3 位非團隊成員從開箱到第一次對話都在 10 分鐘內完成</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -872,18 +936,27 @@
           <t>12/21–12/25</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>大貨生產；中期驗貨</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>12/25–26 香港假期</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr"/>
-      <c r="F15" s="5" t="inlineStr"/>
+      <c r="C15" s="8" t="inlineStr"/>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>大貨生產</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>產量按排期進行</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>中期驗貨（12/25–26 香港假期）</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>中期驗貨抽檢合格</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
@@ -898,24 +971,25 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
+          <t>12/31 大貨完成</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
           <t>大貨完成</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>全部數量完成</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>1/1 假期</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>12/31 大貨完成</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>全部數量完成；中期驗貨合格</t>
-        </is>
-      </c>
+      <c r="G16" s="6" t="inlineStr"/>
     </row>
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -928,18 +1002,27 @@
           <t>1/4–1/8</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>緩衝週：返工、補貨；尾期驗貨</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>客戶確認 App 公開日期</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr"/>
-      <c r="F17" s="5" t="inlineStr"/>
+      <c r="C17" s="8" t="inlineStr"/>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>緩衝週：返工、補貨</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>返工和補貨全部完成</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>尾期驗貨；客戶確認 App 公開日期</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>尾期驗貨（AQL）合格</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="40" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
@@ -954,22 +1037,27 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
+          <t>1/15 出貨</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
           <t>包裝、裝箱、出貨</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>App 公開上架</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>1/15 出貨</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>尾期驗貨合格；出貨清單和序號／MAC 對照表；每台已在系統登記</t>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>出貨清單和序號／MAC 對照表交我方</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>App 公開上架；確認設備登記</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>每台都已在系統登記；三個 App 公開</t>
         </is>
       </c>
     </row>
@@ -984,18 +1072,19 @@
           <t>1/18–1/29</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr"/>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>1/29 送達</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr"/>
+      <c r="E19" s="6" t="inlineStr"/>
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>運送、簽收</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>1/29 送達</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>全部簽收</t>
         </is>
@@ -1004,7 +1093,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>黃色格是關鍵節點和驗收標準：延誤的話，後面的日期會跟著推遲，請提早通知。</t>
+          <t>黃色格是關鍵節點和驗收標準。關鍵節點延誤的話，後面的日期會跟著推遲，請提早通知。</t>
         </is>
       </c>
     </row>
@@ -1017,10 +1106,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -1094,7 +1183,7 @@
           <t>對接方案定案</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>① 網頁和殼的對接清單：藍牙配網、原生登入、推送、麥克風、刪除帳號、深層連結，每項寫明介面、參數、回傳和錯誤
 ② 做殼的同事書面確認
@@ -1118,7 +1207,7 @@
           <t>登入和品牌主題</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>① email 驗證碼登入可用；Google／Apple 登入由殼完成，網頁收得到登入結果
 ② App 內可以刪除帳號
@@ -1142,7 +1231,7 @@
           <t>AI Buddy App 可以內部測試</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>① iPhone 和 Android 都能用藍牙找到玩具、選 Wi-Fi、完成綁定，10 分鐘內做完
 ② 選角色、對話、改設定、解綁都正常
@@ -1166,7 +1255,7 @@
           <t>快活和政協青年聯會 App 頁面完成</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>① 快活：會員綁定、查看記憶、一鍵忘記、選語言（粵／普／英）
 ② 政協青年聯會版：品牌頁面和角色
@@ -1190,7 +1279,7 @@
           <t>功能凍結</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>① 三個 App 全流程通過：安裝 → 登入 → 藍牙配網 → 綁定 → 對話 → 解綁；iOS 和 Android 各至少兩款手機
 ② Wi-Fi 密碼錯、玩具已被別人綁定、斷網時都有清楚提示
@@ -1215,7 +1304,7 @@
           <t>提交商店審核</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>① 上架資料齊全：截圖、描述、私隱政策網址、私隱標籤、審核用測試帳號、玩具示範影片
 ② 三個 App 已提交蘋果和 Google</t>
@@ -1238,7 +1327,7 @@
           <t>通過審核</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>① 三個 App 都通過蘋果和 Google 審核
 ② 如果被拒，修改後重交並通過</t>
@@ -1261,7 +1350,7 @@
           <t>客戶驗收</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>① 馬會、政協青年聯會用正式版走一次完整流程，書面確認
 ② 找 3 位非團隊成員，從開箱到第一次對話都在 10 分鐘內完成
@@ -1285,7 +1374,7 @@
           <t>公開上架</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>① 三個 App 公開，用戶搜尋得到
 ② App 內看得到客服聯絡方式、常見問題、保修條款</t>
@@ -1363,7 +1452,7 @@
           <t>收音</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>距離 1 米正常說話，語音識別正確；和裸板比較不能明顯變差</t>
         </is>
@@ -1380,7 +1469,7 @@
           <t>喇叭</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>隔著布料的響度和清晰度；最大音量不破音、不震動</t>
         </is>
@@ -1397,7 +1486,7 @@
           <t>按鍵</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>隔著布料／徽章按得到，小朋友按得動，回彈清楚</t>
         </is>
@@ -1414,7 +1503,7 @@
           <t>Wi-Fi</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>裝進公仔後訊號強度，和裸板比較</t>
         </is>
@@ -1431,7 +1520,7 @@
           <t>充電</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>USB-C 插得進，充電時燈號看得到</t>
         </is>
@@ -1448,7 +1537,7 @@
           <t>燈號</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>低電紅燈從外面看得到（或確定不外露）</t>
         </is>
@@ -1465,7 +1554,7 @@
           <t>跌落</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>1 米跌落，零件不脫落，機芯盒不鬆脫</t>
         </is>
@@ -1482,7 +1571,7 @@
           <t>小零件與尖角</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>眼睛、徽章、配件拉力測試；沒有尖角和可吞食的小零件</t>
         </is>
@@ -1499,7 +1588,7 @@
           <t>拆裝</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>機芯盒能取出維修，縫口或拉鍊位置合理</t>
         </is>

</xml_diff>

<commit_message>
Plan web, tool calls, RAG, admin, testing and UAT, not just the apps.
The factory workbook's app sheet becomes '軟件開發與測試': nineteen dated
steps across seven workstreams (web pages, app shell and store, tool
calls, the HKJC RAG knowledge base, admin and the three stacks, internal
and system testing, client UAT), each with checkable acceptance
criteria. roadmap.md carries the same table with tracker IDs, and the
weekly table now names system testing (W7–W8) and client UAT (W9–W10).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/毛公仔打版與量產時間表_草案v0.5.xlsx
+++ b/docs/毛公仔打版與量產時間表_草案v0.5.xlsx
@@ -8,11 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="時間表" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App 開發與上架" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="軟件開發與測試" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="樣品測試項目" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'時間表'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'軟件開發與測試'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -82,7 +83,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -104,11 +105,44 @@
         <color rgb="00C9CED6"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9CED6"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9CED6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C9CED6"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9CED6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C9CED6"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C9CED6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -131,6 +165,11 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -777,7 +816,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="56" customHeight="1">
+    <row r="11" ht="72" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>W7</t>
@@ -805,7 +844,7 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>確認產前樣、下大貨單；出廠韌體交電路板供應商；App 功能凍結</t>
+          <t>確認產前樣、下大貨單；出廠韌體交電路板供應商；網頁和 App 功能凍結，系統測試開始</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -842,12 +881,12 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>交燒錄自檢工位和作業指導書；App 提交蘋果和 Google 審核</t>
+          <t>交燒錄自檢工位和作業指導書；App 提交蘋果和 Google 審核；系統測試</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>工位在工廠試跑 10 台全部通過；三個 App 已提交，上架資料齊全</t>
+          <t>工位在工廠試跑 10 台全部通過；三個 App 已提交，上架資料齊全；系統測試和壓測通過</t>
         </is>
       </c>
     </row>
@@ -879,7 +918,7 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>全檢試產品；App 審核（預留被拒重交的時間）</t>
+          <t>全檢試產品；App 審核（預留被拒重交的時間）；客戶 UAT 開始</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -916,12 +955,12 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>App 上架但不公開，客戶驗收</t>
+          <t>客戶 UAT 完成；App 上架但不公開</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>客戶書面確認 App；3 位非團隊成員從開箱到第一次對話都在 10 分鐘內完成</t>
+          <t>客戶 UAT 書面簽收，嚴重問題 0 個；3 位非團隊成員從開箱到第一次對話都在 10 分鐘內完成</t>
         </is>
       </c>
     </row>
@@ -1122,269 +1161,533 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="64" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>App 開發與上架：里程碑和驗收標準</t>
+          <t>軟件開發與測試：網頁、App、Tool call、RAG、後台、測試、UAT</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>網頁 App 包在原生殼裡，三個品牌各一個 App。殼過審後，網頁畫面可以繼續更新，不用重新送審。</t>
+          <t>網頁 App 包在原生殼裡，三個品牌各一個 App、各一套系統。殼過審後，網頁畫面可以繼續更新，不用重新送審。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
+          <t>工作線</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
           <t>週次</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>日期</t>
-        </is>
-      </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>里程碑</t>
+          <t>完成日期</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
+          <t>內容</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
           <t>驗收標準（全部做到才算完成）</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="72" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>W2</t>
+    <row r="5" ht="56" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>網頁</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
+          <t>W1–W3</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>10/30</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>共用基礎：品牌主題、App 內登入、刪除帳號</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>三個品牌的顏色、logo、文案顯示正確，畫面不閃；email 驗證碼登入、Google／Apple 登入（由殼完成）、App 內刪除帳號都可用</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>W3–W4</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>11/6</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>AI Buddy 網頁：配網、綁定、角色、設定、家長控制</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>iPhone 和 Android 上 10 分鐘內完成藍牙配網和綁定；選角色、對話、改設定、解綁、家長鎖、每日上限都正常</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>W4–W6</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>11/20</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>快活和政協青年聯會網頁</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>快活：會員綁定、查看記憶、一鍵忘記、選語言（粵／普／英）；政協青年聯會版：品牌頁面和角色</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="56" customHeight="1">
+      <c r="A8" s="12" t="n"/>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>11/27</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>功能凍結</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>三個品牌全流程通過：安裝 → 登入 → 配網 → 綁定 → 對話 → 解綁，iOS 和 Android 各至少兩款手機；Wi-Fi 密碼錯、玩具已被綁定、斷網時都有清楚提示</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="56" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>App 殼與上架</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>W1–W2</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
           <t>10/23</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>對接方案定案</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>① 網頁和殼的對接清單：藍牙配網、原生登入、推送、麥克風、刪除帳號、深層連結，每項寫明介面、參數、回傳和錯誤
-② 做殼的同事書面確認
-③ 三個 App 的名稱、圖示、bundle id 定好</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="72" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>W3</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>網頁和殼的對接方案</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>對接清單（藍牙配網、原生登入、推送、麥克風、刪除帳號、深層連結）逐項寫明介面和錯誤，做殼的同事書面確認；三個 App 的名稱、圖示、bundle id 定好</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="56" customHeight="1">
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>W3–W6</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>11/20</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>殼開發、測試版</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>三個 App 的測試版可以安裝（TestFlight、Google 內部測試）；藍牙、登入、推送（玩具上線、低電）可用；連續使用 30 分鐘不閃退</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="56" customHeight="1">
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>W8–W9</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>12/11</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>提交審核、通過審核</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>11/30 提交，上架資料齊全（截圖、私隱政策、私隱標籤、審核用帳號、玩具示範影片）；12/11 前三個 App 通過蘋果和 Google 審核</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>1/15</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>公開上架</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>三個 App 公開，用戶搜尋得到；App 內看得到客服、常見問題、保修條款</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="56" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Tool call</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>W2–W3</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>10/30</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>登入和品牌主題</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>① email 驗證碼登入可用；Google／Apple 登入由殼完成，網頁收得到登入結果
-② App 內可以刪除帳號
-③ 三個品牌各自的顏色、logo、文案顯示正確，畫面不閃</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="72" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>工具清單和設計</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>定好語音助手可以調用的工具（建議：天氣、日期和節日、調音量、結束對話、快活的賽事資料查詢），每個工具的觸發說法和回覆方式，以及每個品牌允許哪些工具</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>W4–W6</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>11/20</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>開發和測試</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>每個工具用真實語音觸發 20 次，成功率 ≥ 95%；不相關的話不會誤觸發；首字延遲增加不超過 300 毫秒</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>RAG 知識庫（快活）</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>11/6</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>AI Buddy App 可以內部測試</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>① iPhone 和 Android 都能用藍牙找到玩具、選 Wi-Fi、完成綁定，10 分鐘內做完
-② 選角色、對話、改設定、解綁都正常
-③ 家長控制（家長鎖、每日上限）可用</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="56" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>收資料、入庫流程</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>馬會第一批資料已收到；入庫、版本、審批流程跑通一次</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>W5–W8</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>12/4</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>檢索和回答</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>100 條測試問題答對率 ≥ 90%；知識庫沒有的內容會說不肯定並建議查詢；問貼士、賠率、賽果預測 100% 婉拒</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="12" t="n"/>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>W9–W11</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>12/25</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>馬會審核 v1</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>馬會書面批准 v1；每一版都有審批記錄；更新知識庫不用重新燒錄玩具</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="56" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>後台管理</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>W3–W6</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>11/20</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>快活和政協青年聯會 App 頁面完成</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>① 快活：會員綁定、查看記憶、一鍵忘記、選語言（粵／普／英）
-② 政協青年聯會版：品牌頁面和角色
-③ 三個 App 都有測試版可以安裝（TestFlight、Google 內部測試）</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="88" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>管理功能</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>內容管理員：上載知識庫並送審、發佈角色；超級管理員：看設備最後上線、韌體版本、錯誤，發佈 OTA，解綁和換機；任何管理員都看不到對話內容</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="12" t="n"/>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>W6–W8</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>12/4</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>三個品牌各自一套系統</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>三套各自上線，冒煙測試（登入、對話、OTA 檢查）通過；部署腳本一次跑完三套；一套停機不影響另外兩套</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>測試</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>W4–W7</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>11/27</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>功能凍結</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>① 三個 App 全流程通過：安裝 → 登入 → 藍牙配網 → 綁定 → 對話 → 解綁；iOS 和 Android 各至少兩款手機
-② Wi-Fi 密碼錯、玩具已被別人綁定、斷網時都有清楚提示
-③ 推送收得到：玩具第一次上線、低電提醒
-④ 連續使用 30 分鐘不閃退</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="56" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>11/30</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>提交商店審核</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>① 上架資料齊全：截圖、描述、私隱政策網址、私隱標籤、審核用測試帳號、玩具示範影片
-② 三個 App 已提交蘋果和 Google</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>W9</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>12/11</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>通過審核</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>① 三個 App 都通過蘋果和 Google 審核
-② 如果被拒，修改後重交並通過</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="56" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>W10</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>內部測試（20 台、4 週）</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>每週記錄對話輪數、首字延遲、每台成本、安全事件；第 4 週出測試報告</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="12" t="n"/>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>W7–W8</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>12/4</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>系統測試</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>全流程測試通過；按 3,000 台規模壓測（150–300 個同時對話）通過；安全測試通過；嚴重問題 0 個</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="56" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>W9–W10</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
         <is>
           <t>12/18</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>客戶驗收</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>① 馬會、政協青年聯會用正式版走一次完整流程，書面確認
-② 找 3 位非團隊成員，從開箱到第一次對話都在 10 分鐘內完成
-③ App 已上架但不公開</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>W14</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>1/15</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>公開上架</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>① 三個 App 公開，用戶搜尋得到
-② App 內看得到客服聯絡方式、常見問題、保修條款</t>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>客戶 UAT（用試產機和正式版 App）</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>按 UAT 清單逐項測完；馬會、政協青年聯會書面簽收；嚴重問題 0 個，其他問題都有處理日期；3 位非團隊成員從開箱到第一次對話都在 10 分鐘內完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="12" t="n"/>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>1/8</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>上線前最後確認</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>UAT 遺留問題全部處理；正式環境凍結，只修 bug；監控和告警正常</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
+  <mergeCells count="9">
+    <mergeCell ref="A9:A12"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A5:A8"/>
+    <mergeCell ref="A18:A19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Name who owns each software step: Neo for the app shell.
The software sheet and roadmap table gain an owner column. Neo builds
the native shell (bridge spec with us, test builds, store submission,
release); everything else in software is the user plus Claude, shown as
我方軟件. HKJC supplies and approves the RAG data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/毛公仔打版與量產時間表_草案v0.5.xlsx
+++ b/docs/毛公仔打版與量產時間表_草案v0.5.xlsx
@@ -659,12 +659,12 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>審 3D 圖；決定電路板改不改；定好 App 和網頁的對接方式</t>
+          <t>審 3D 圖；決定電路板改不改；和 Neo 定好 App 殼和網頁的對接方式</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>2 個工作天內回覆 3D 圖意見；改不改板有書面結論；對接清單由做殼的同事確認</t>
+          <t>2 個工作天內回覆 3D 圖意見；改不改板有書面結論；對接清單由 Neo 確認</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>交燒錄自檢工位和作業指導書；App 提交蘋果和 Google 審核；系統測試</t>
+          <t>交燒錄自檢工位和作業指導書；Neo 提交三個 App 給蘋果和 Google 審核；系統測試</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1161,14 +1161,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="64" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1181,7 +1182,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>網頁 App 包在原生殼裡，三個品牌各一個 App、各一套系統。殼過審後，網頁畫面可以繼續更新，不用重新送審。</t>
+          <t>網頁 App 包在原生殼裡，三個品牌各一個 App、各一套系統。殼由 Neo 負責；「我方軟件」是網頁、後台、語音系統和韌體。殼過審後，網頁畫面可以繼續更新，不用重新送審。</t>
         </is>
       </c>
     </row>
@@ -1203,10 +1204,15 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
+          <t>負責</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
           <t>內容</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>驗收標準（全部做到才算完成）</t>
         </is>
@@ -1228,12 +1234,17 @@
           <t>10/30</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>我方軟件</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>共用基礎：品牌主題、App 內登入、刪除帳號</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>三個品牌的顏色、logo、文案顯示正確，畫面不閃；email 驗證碼登入、Google／Apple 登入（由殼完成）、App 內刪除帳號都可用</t>
         </is>
@@ -1251,12 +1262,17 @@
           <t>11/6</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>我方軟件</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>AI Buddy 網頁：配網、綁定、角色、設定、家長控制</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>iPhone 和 Android 上 10 分鐘內完成藍牙配網和綁定；選角色、對話、改設定、解綁、家長鎖、每日上限都正常</t>
         </is>
@@ -1274,12 +1290,17 @@
           <t>11/20</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>我方軟件</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>快活和政協青年聯會網頁</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>快活：會員綁定、查看記憶、一鍵忘記、選語言（粵／普／英）；政協青年聯會版：品牌頁面和角色</t>
         </is>
@@ -1297,12 +1318,17 @@
           <t>11/27</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>我方軟件</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>功能凍結</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>三個品牌全流程通過：安裝 → 登入 → 配網 → 綁定 → 對話 → 解綁，iOS 和 Android 各至少兩款手機；Wi-Fi 密碼錯、玩具已被綁定、斷網時都有清楚提示</t>
         </is>
@@ -1324,12 +1350,17 @@
           <t>10/23</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Neo、我方軟件</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>網頁和殼的對接方案</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>對接清單（藍牙配網、原生登入、推送、麥克風、刪除帳號、深層連結）逐項寫明介面和錯誤，做殼的同事書面確認；三個 App 的名稱、圖示、bundle id 定好</t>
         </is>
@@ -1347,12 +1378,17 @@
           <t>11/20</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Neo</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>殼開發、測試版</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>三個 App 的測試版可以安裝（TestFlight、Google 內部測試）；藍牙、登入、推送（玩具上線、低電）可用；連續使用 30 分鐘不閃退</t>
         </is>
@@ -1370,12 +1406,17 @@
           <t>12/11</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Neo（客戶提供開發者帳號）</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>提交審核、通過審核</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>11/30 提交，上架資料齊全（截圖、私隱政策、私隱標籤、審核用帳號、玩具示範影片）；12/11 前三個 App 通過蘋果和 Google 審核</t>
         </is>
@@ -1393,12 +1434,17 @@
           <t>1/15</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Neo</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>公開上架</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>三個 App 公開，用戶搜尋得到；App 內看得到客服、常見問題、保修條款</t>
         </is>
@@ -1420,12 +1466,17 @@
           <t>10/30</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>我方軟件</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>工具清單和設計</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>定好語音助手可以調用的工具（建議：天氣、日期和節日、調音量、結束對話、快活的賽事資料查詢），每個工具的觸發說法和回覆方式，以及每個品牌允許哪些工具</t>
         </is>
@@ -1443,18 +1494,23 @@
           <t>11/20</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>我方軟件</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>開發和測試</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>每個工具用真實語音觸發 20 次，成功率 ≥ 95%；不相關的話不會誤觸發；首字延遲增加不超過 300 毫秒</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
+    <row r="15" ht="40" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
           <t>RAG 知識庫（快活）</t>
@@ -1470,12 +1526,17 @@
           <t>11/6</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>馬會提供資料；我方軟件</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>收資料、入庫流程</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>馬會第一批資料已收到；入庫、版本、審批流程跑通一次</t>
         </is>
@@ -1493,12 +1554,17 @@
           <t>12/4</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>我方軟件</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>檢索和回答</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>100 條測試問題答對率 ≥ 90%；知識庫沒有的內容會說不肯定並建議查詢；問貼士、賠率、賽果預測 100% 婉拒</t>
         </is>
@@ -1516,12 +1582,17 @@
           <t>12/25</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>馬會審核；我方軟件修改</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>馬會審核 v1</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>馬會書面批准 v1；每一版都有審批記錄；更新知識庫不用重新燒錄玩具</t>
         </is>
@@ -1543,12 +1614,17 @@
           <t>11/20</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>我方軟件</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>管理功能</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>內容管理員：上載知識庫並送審、發佈角色；超級管理員：看設備最後上線、韌體版本、錯誤，發佈 OTA，解綁和換機；任何管理員都看不到對話內容</t>
         </is>
@@ -1566,12 +1642,17 @@
           <t>12/4</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>我方軟件</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>三個品牌各自一套系統</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>三套各自上線，冒煙測試（登入、對話、OTA 檢查）通過；部署腳本一次跑完三套；一套停機不影響另外兩套</t>
         </is>
@@ -1593,12 +1674,17 @@
           <t>11/27</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>我方全體</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>內部測試（20 台、4 週）</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>每週記錄對話輪數、首字延遲、每台成本、安全事件；第 4 週出測試報告</t>
         </is>
@@ -1616,12 +1702,17 @@
           <t>12/4</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>我方軟件</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>系統測試</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>全流程測試通過；按 3,000 台規模壓測（150–300 個同時對話）通過；安全測試通過；嚴重問題 0 個</t>
         </is>
@@ -1643,12 +1734,17 @@
           <t>12/18</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>馬會、政協青年聯會；我方</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>客戶 UAT（用試產機和正式版 App）</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>按 UAT 清單逐項測完；馬會、政協青年聯會書面簽收；嚴重問題 0 個，其他問題都有處理日期；3 位非團隊成員從開箱到第一次對話都在 10 分鐘內完成</t>
         </is>
@@ -1666,12 +1762,17 @@
           <t>1/8</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>我方軟件</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>上線前最後確認</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>UAT 遺留問題全部處理；正式環境凍結，只修 bug；監控和告警正常</t>
         </is>
@@ -1679,12 +1780,12 @@
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="A2:F2"/>
     <mergeCell ref="A9:A12"/>
-    <mergeCell ref="A2:E2"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A15:A17"/>
-    <mergeCell ref="A1:E1"/>
     <mergeCell ref="A20:A21"/>
     <mergeCell ref="A5:A8"/>
     <mergeCell ref="A18:A19"/>

</xml_diff>